<commit_message>
The halal promise without "no pork, no alcohol"
The owner wants that phrase out of every wording. The trust line, voice rule, halal-seeker message and the two
Halal wordings now say "100% halal meat from certified suppliers"; the strategy workbook is regenerated. The bank
upsert on item + headline updates the two live wordings at the next boot.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/calendar/Fuadijan-Strategy-2026-11.xlsx
+++ b/calendar/Fuadijan-Strategy-2026-11.xlsx
@@ -2712,7 +2712,7 @@
       </c>
       <c s="0" r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">No pork · No alcohol · Certified suppliers</t>
+          <t xml:space="preserve">Fresh meat · Certified suppliers · Every dish</t>
         </is>
       </c>
     </row>
@@ -3024,12 +3024,12 @@
       </c>
       <c s="0" r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">100% halal meat from certified suppliers, no pork, no alcohol — ever.</t>
+          <t xml:space="preserve">100% halal meat from certified suppliers — always.</t>
         </is>
       </c>
       <c s="0" r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Our halal promise: 100% halal meat from certified suppliers, no pork, no alcohol — ever. Certificates on display in store and in our Halal highlight. Eat with peace of mind.
+          <t xml:space="preserve">Our halal promise: 100% halal meat from certified suppliers — always. Certificates on display in store and in our Halal highlight. Eat with peace of mind.
 #HalalFood #SydneyHalal #MuslimSydney</t>
         </is>
       </c>

</xml_diff>

<commit_message>
FRESH POUR and SAVE ROOM: series for drinks and sweets
The menu's Beverages and Sweets had no series, so a carrot juice or a gulab jamun fell through to ROOTED IN
TRADITION. FRESH POUR (brand footer) joins the registry beside the existing SAVE ROOM; the series picker knows
drink and sweet words; and a product's menu category now suggests its series: Create preselects it (and marks
it "suggested"), /custom starts from it. The strategy gains the two roles (pairing, finish), hashtag sets for
drinks and sweets, a pairing caption pattern, five posters and two captions for the bank (38 wordings), and two
shot-list lines; the workbook is regenerated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/calendar/Fuadijan-Strategy-2026-11.xlsx
+++ b/calendar/Fuadijan-Strategy-2026-11.xlsx
@@ -2845,364 +2845,502 @@
     <row r="16">
       <c s="0" r="A16" t="inlineStr">
         <is>
+          <t xml:space="preserve">Carrot Juice</t>
+        </is>
+      </c>
+      <c s="0" r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poured cold.
+Drunk fast.</t>
+        </is>
+      </c>
+      <c s="0" r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carrot juice beside the plate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c s="0" r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sugarcane Juice</t>
+        </is>
+      </c>
+      <c s="0" r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sugarcane,
+over ice</t>
+        </is>
+      </c>
+      <c s="0" r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The grill's best friend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c s="0" r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mango Lassi</t>
+        </is>
+      </c>
+      <c s="0" r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cool the
+karahi down</t>
+        </is>
+      </c>
+      <c s="0" r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mango lassi, thick and cold.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c s="0" r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulab Jamun</t>
+        </is>
+      </c>
+      <c s="0" r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save
+room.</t>
+        </is>
+      </c>
+      <c s="0" r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulab jamun, in syrup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c s="0" r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kheer</t>
+        </is>
+      </c>
+      <c s="0" r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The sweet
+finish</t>
+        </is>
+      </c>
+      <c s="0" r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kheer, by the bowl, for the table.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c s="0" r="A21" t="inlineStr">
+        <is>
           <t xml:space="preserve">Chicken Karahi</t>
         </is>
       </c>
-      <c s="0" r="B16" t="inlineStr">
+      <c s="0" r="B21" t="inlineStr">
         <is>
           <t xml:space="preserve">Cooked fresh
 when you order</t>
         </is>
       </c>
-      <c s="0" r="C16" t="inlineStr">
+      <c s="0" r="C21" t="inlineStr">
         <is>
           <t xml:space="preserve">Tomatoes, ginger, green chilli, and a wok that's seen a thousand Friday nights.</t>
         </is>
       </c>
-      <c s="0" r="D16" t="inlineStr">
+      <c s="0" r="D21" t="inlineStr">
         <is>
           <t xml:space="preserve">Tomatoes, ginger, green chilli, and a wok that's seen a thousand Friday nights. Our Chicken Karahi is cooked fresh when you order — never sitting in a tray. 100% halal.
 #ChickenKarahi #HalalSydney #AuburnEats</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c s="0" r="A17" t="inlineStr">
+    <row r="22">
+      <c s="0" r="A22" t="inlineStr">
         <is>
           <t xml:space="preserve">Chapli Kebab Day</t>
         </is>
       </c>
-      <c s="0" r="B17" t="inlineStr">
+      <c s="0" r="B22" t="inlineStr">
         <is>
           <t xml:space="preserve">It's Chapli
 Kebab Day</t>
         </is>
       </c>
-      <c s="0" r="C17" t="inlineStr">
+      <c s="0" r="C22" t="inlineStr">
         <is>
           <t xml:space="preserve">Hand-pressed beef, crushed coriander, pomegranate, a crisp edge and a juicy middle.</t>
         </is>
       </c>
-      <c s="0" r="D17" t="inlineStr">
+      <c s="0" r="D22" t="inlineStr">
         <is>
           <t xml:space="preserve">It's Chapli Kebab Day 🔥 Hand-pressed beef, crushed coriander, pomegranate, a crisp edge and a juicy middle. First Friday of every month — today only, [offer]. Tag the friend who's never tried chapli.
 #ChapliKebab #PakistaniBBQ #SydneyFood</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c s="0" r="A18" t="inlineStr">
+    <row r="23">
+      <c s="0" r="A23" t="inlineStr">
         <is>
           <t xml:space="preserve">Chicken Tikka</t>
         </is>
       </c>
-      <c s="0" r="B18" t="inlineStr">
+      <c s="0" r="B23" t="inlineStr">
         <is>
           <t xml:space="preserve">Fresh off
 the grill</t>
         </is>
       </c>
-      <c s="0" r="C18" t="inlineStr">
+      <c s="0" r="C23" t="inlineStr">
         <is>
           <t xml:space="preserve">Chicken tikka, seekh kebab, and that smoky char you can't fake.</t>
         </is>
       </c>
-      <c s="0" r="D18" t="inlineStr">
+      <c s="0" r="D23" t="inlineStr">
         <is>
           <t xml:space="preserve">Fresh off the grill, straight to your table. Chicken tikka, seekh kebab, and that smoky char you can't fake. Who's coming tonight?
 #PakistaniBBQ #ChickenTikka #AuburnEats</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c s="0" r="A19" t="inlineStr">
+    <row r="24">
+      <c s="0" r="A24" t="inlineStr">
         <is>
           <t xml:space="preserve">Karahi Night</t>
         </is>
       </c>
-      <c s="0" r="B19" t="inlineStr">
+      <c s="0" r="B24" t="inlineStr">
         <is>
           <t xml:space="preserve">Wednesday =
 Karahi Night</t>
         </is>
       </c>
-      <c s="0" r="C19" t="inlineStr">
+      <c s="0" r="C24" t="inlineStr">
         <is>
           <t xml:space="preserve">Bring the family, we'll bring the karahi.</t>
         </is>
       </c>
-      <c s="0" r="D19" t="inlineStr">
+      <c s="0" r="D24" t="inlineStr">
         <is>
           <t xml:space="preserve">Wednesday = Karahi Night 🍲 [Offer], 5–10pm. Bring the family, we'll bring the karahi.
 #KarahiNight #Karahi #WesternSydney</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c s="0" r="A20" t="inlineStr">
+    <row r="25">
+      <c s="0" r="A25" t="inlineStr">
         <is>
           <t xml:space="preserve">Reviews</t>
         </is>
       </c>
-      <c s="0" r="B20" t="inlineStr">
+      <c s="0" r="B25" t="inlineStr">
         <is>
           <t xml:space="preserve">This is why
 we cook to order</t>
         </is>
       </c>
-      <c s="0" r="C20" t="inlineStr">
+      <c s="0" r="C25" t="inlineStr">
         <is>
           <t xml:space="preserve">Thank you!</t>
         </is>
       </c>
-      <c s="0" r="D20" t="inlineStr">
+      <c s="0" r="D25" t="inlineStr">
         <is>
           <t xml:space="preserve">"[Short real review line]" — [Name] ⭐⭐⭐⭐⭐ Thank you! This is why we cook everything to order.
 #Fuadijan #HalalFood</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c s="0" r="A21" t="inlineStr">
+    <row r="26">
+      <c s="0" r="A26" t="inlineStr">
         <is>
           <t xml:space="preserve">Family Feast</t>
         </is>
       </c>
-      <c s="0" r="B21" t="inlineStr">
+      <c s="0" r="B26" t="inlineStr">
         <is>
           <t xml:space="preserve">Big table?
 Big platter.</t>
         </is>
       </c>
-      <c s="0" r="C21" t="inlineStr">
+      <c s="0" r="C26" t="inlineStr">
         <is>
           <t xml:space="preserve">Tikka, seekh, karahi, naan and something for the kids. Easy parking.</t>
         </is>
       </c>
-      <c s="0" r="D21" t="inlineStr">
+      <c s="0" r="D26" t="inlineStr">
         <is>
           <t xml:space="preserve">Big table? Big platter. Easy parking. Our family feast feeds [4–6] with tikka, seekh, karahi, naan and something for the kids. Book your table: [phone]
 #FamilyDinnerSydney #HalalSydney</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c s="0" r="A22" t="inlineStr">
+    <row r="27">
+      <c s="0" r="A27" t="inlineStr">
         <is>
           <t xml:space="preserve">Student Combo</t>
         </is>
       </c>
-      <c s="0" r="B22" t="inlineStr">
+      <c s="0" r="B27" t="inlineStr">
         <is>
           <t xml:space="preserve">Exams are hard.
 Dinner shouldn't be.</t>
         </is>
       </c>
-      <c s="0" r="C22" t="inlineStr">
+      <c s="0" r="C27" t="inlineStr">
         <is>
           <t xml:space="preserve">Student combo, Tuesdays, with student ID.</t>
         </is>
       </c>
-      <c s="0" r="D22" t="inlineStr">
+      <c s="0" r="D27" t="inlineStr">
         <is>
           <t xml:space="preserve">Exams are hard. Dinner shouldn't be. Student combo: [item] + chips + drink for $[X] with student ID, Tuesdays.
 #SydneyStudents #CheapEatsSydney #UniLife</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c s="0" r="A23" t="inlineStr">
+    <row r="28">
+      <c s="0" r="A28" t="inlineStr">
         <is>
           <t xml:space="preserve">Halal</t>
         </is>
       </c>
-      <c s="0" r="B23" t="inlineStr">
+      <c s="0" r="B28" t="inlineStr">
         <is>
           <t xml:space="preserve">Our halal
 promise</t>
         </is>
       </c>
-      <c s="0" r="C23" t="inlineStr">
+      <c s="0" r="C28" t="inlineStr">
         <is>
           <t xml:space="preserve">100% halal meat from certified suppliers — always.</t>
         </is>
       </c>
-      <c s="0" r="D23" t="inlineStr">
+      <c s="0" r="D28" t="inlineStr">
         <is>
           <t xml:space="preserve">Our halal promise: 100% halal meat from certified suppliers — always. Certificates on display in store and in our Halal highlight. Eat with peace of mind.
 #HalalFood #SydneyHalal #MuslimSydney</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c s="0" r="A24" t="inlineStr">
+    <row r="29">
+      <c s="0" r="A29" t="inlineStr">
         <is>
           <t xml:space="preserve">Behind Fuadijan</t>
         </is>
       </c>
-      <c s="0" r="B24" t="inlineStr">
+      <c s="0" r="B29" t="inlineStr">
         <is>
           <t xml:space="preserve">There isn't
 a shortcut</t>
         </is>
       </c>
-      <c s="0" r="C24" t="inlineStr">
+      <c s="0" r="C29" t="inlineStr">
         <is>
           <t xml:space="preserve">The marinade's been going since last night; the grill's warming up.</t>
         </is>
       </c>
-      <c s="0" r="D24" t="inlineStr">
+      <c s="0" r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">9am. The marinade's been going since last night, the grill's warming up, and the naan dough is resting. That's the secret — there isn't a shortcut.
 #FuadijanKitchen #PakistaniFood</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c s="0" r="A25" t="inlineStr">
+    <row r="30">
+      <c s="0" r="A30" t="inlineStr">
         <is>
           <t xml:space="preserve">Burgers</t>
         </is>
       </c>
-      <c s="0" r="B25" t="inlineStr">
+      <c s="0" r="B30" t="inlineStr">
         <is>
           <t xml:space="preserve">Karahi for you,
 burger for them</t>
         </is>
       </c>
-      <c s="0" r="C25" t="inlineStr">
+      <c s="0" r="C30" t="inlineStr">
         <is>
           <t xml:space="preserve">Not everyone at the table wants karahi — and that's fine.</t>
         </is>
       </c>
-      <c s="0" r="D25" t="inlineStr">
+      <c s="0" r="D30" t="inlineStr">
         <is>
           <t xml:space="preserve">Not everyone at the table wants karahi — and that's fine. Our [burger name]: [patty], [sauce], toasted bun, 100% halal. Karahi for you, burger for them.
 #HalalBurger #AuburnEats #SydneyEats</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c s="0" r="A26" t="inlineStr">
+    <row r="31">
+      <c s="0" r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carrot Juice</t>
+        </is>
+      </c>
+      <c s="0" r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Poured cold.
+Drunk fast.</t>
+        </is>
+      </c>
+      <c s="0" r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carrot juice beside the plate.</t>
+        </is>
+      </c>
+      <c s="0" r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carrot juice, poured cold, beside a plate from the grill. Ask for it with your order, or on its own at the counter.
+#FreshJuice #CarrotJuice #AuburnEats</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c s="0" r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulab Jamun</t>
+        </is>
+      </c>
+      <c s="0" r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Save
+room.</t>
+        </is>
+      </c>
+      <c s="0" r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulab jamun, in syrup.</t>
+        </is>
+      </c>
+      <c s="0" r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gulab jamun in syrup: how the family table ends. Add it to any order, and share it if you can.
+#GulabJamun #SydneyDesserts #PakistaniSweets</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c s="0" r="A33" t="inlineStr">
         <is>
           <t xml:space="preserve">Family Feast</t>
         </is>
       </c>
-      <c s="0" r="B26" t="inlineStr">
+      <c s="0" r="B33" t="inlineStr">
         <is>
           <t xml:space="preserve">Summer feasts,
 easy parking</t>
         </is>
       </c>
-      <c s="0" r="C26" t="inlineStr">
+      <c s="0" r="C33" t="inlineStr">
         <is>
           <t xml:space="preserve">Family platters all holidays · Easy parking</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c s="0" r="A27" t="inlineStr">
+    <row r="34">
+      <c s="0" r="A34" t="inlineStr">
         <is>
           <t xml:space="preserve">Pakistan Day</t>
         </is>
       </c>
-      <c s="0" r="B27" t="inlineStr">
+      <c s="0" r="B34" t="inlineStr">
         <is>
           <t xml:space="preserve">Taste of
 Pakistan</t>
         </is>
       </c>
-      <c s="0" r="C27" t="inlineStr">
+      <c s="0" r="C34" t="inlineStr">
         <is>
           <t xml:space="preserve">23 March · Tasting plate</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c s="0" r="A28" t="inlineStr">
+    <row r="35">
+      <c s="0" r="A35" t="inlineStr">
         <is>
           <t xml:space="preserve">Student Combo</t>
         </is>
       </c>
-      <c s="0" r="B28" t="inlineStr">
+      <c s="0" r="B35" t="inlineStr">
         <is>
           <t xml:space="preserve">Your new
 local</t>
         </is>
       </c>
-      <c s="0" r="C28" t="inlineStr">
+      <c s="0" r="C35" t="inlineStr">
         <is>
           <t xml:space="preserve">Student Night every Tuesday · Show ID</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c s="0" r="A29" t="inlineStr">
+    <row r="36">
+      <c s="0" r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">Eid</t>
         </is>
       </c>
-      <c s="0" r="B29" t="inlineStr">
+      <c s="0" r="B36" t="inlineStr">
         <is>
           <t xml:space="preserve">Eid al-Adha
 Mubarak</t>
         </is>
       </c>
-      <c s="0" r="C29" t="inlineStr">
+      <c s="0" r="C36" t="inlineStr">
         <is>
           <t xml:space="preserve">Lamb karahi special · Catering · Open for Eid lunch</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c s="0" r="A30" t="inlineStr">
+    <row r="37">
+      <c s="0" r="A37" t="inlineStr">
         <is>
           <t xml:space="preserve">Pakistan Day</t>
         </is>
       </c>
-      <c s="0" r="B30" t="inlineStr">
+      <c s="0" r="B37" t="inlineStr">
         <is>
           <t xml:space="preserve">14 August
 at Fuadijan</t>
         </is>
       </c>
-      <c s="0" r="C30" t="inlineStr">
+      <c s="0" r="C37" t="inlineStr">
         <is>
           <t xml:space="preserve">Community night · Green-themed desserts</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c s="0" r="A31" t="inlineStr">
+    <row r="38">
+      <c s="0" r="A38" t="inlineStr">
         <is>
           <t xml:space="preserve">Student Combo</t>
         </is>
       </c>
-      <c s="0" r="B31" t="inlineStr">
+      <c s="0" r="B38" t="inlineStr">
         <is>
           <t xml:space="preserve">Student Night
 is back</t>
         </is>
       </c>
-      <c s="0" r="C31" t="inlineStr">
+      <c s="0" r="C38" t="inlineStr">
         <is>
           <t xml:space="preserve">Tuesdays · Show ID</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c s="0" r="A32" t="inlineStr">
+    <row r="39">
+      <c s="0" r="A39" t="inlineStr">
         <is>
           <t xml:space="preserve">Creator Night</t>
         </is>
       </c>
-      <c s="0" r="B32" t="inlineStr">
+      <c s="0" r="B39" t="inlineStr">
         <is>
           <t xml:space="preserve">Creator
 Tasting Night</t>
         </is>
       </c>
-      <c s="0" r="C32" t="inlineStr">
+      <c s="0" r="C39" t="inlineStr">
         <is>
           <t xml:space="preserve">Fuadijan Grill · By invitation</t>
         </is>

</xml_diff>